<commit_message>
Fix security: remove real system schema and protocol number from samples
[generate_sample_data.py]
- mg_donor_info:KBN_DONOR/SEX/BIRTH_YEAR/BIRTH_MONTH → donor_code/sex/birth_year/birth_month (실제 DB 필드명 제거)
- 슈프림 시트명 1004-037-315 → DEMO-000-000 (실제 프로토콜 번호 제거)
- Master_DB_샘플에서 생성ID 컬럼 제거 (값에서 내부 키 형식 노출 방지)
- build_internal_key/parse_personal_no import 제거

[clinical_data_qc.py]
- _read_hubis_fix() docstring에서 실제 필드명 제거
- run_rid_matching(): COL_GEN_ID 누락 시 KeyError 방어 처리 추가

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/Master_DB_샘플.xlsx
+++ b/sample_data/Master_DB_샘플.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,11 +451,6 @@
           <t>접수일자</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>생성ID</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -486,11 +481,6 @@
           <t>2024-03-15</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>M199305김20240315</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -521,11 +511,6 @@
           <t>2024-03-15</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>F197511이20240315</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -556,11 +541,6 @@
           <t>2024-03-18</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>M198207박20240318</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -591,11 +571,6 @@
           <t>2024-03-16</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>F199004최20240316</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -626,11 +601,6 @@
           <t>2024-03-16</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>M200109정20240316</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -661,11 +631,6 @@
           <t>2024-03-17</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>F195512강20240317</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -696,11 +661,6 @@
           <t>2024-03-17</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>M197906조20240317</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -729,11 +689,6 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>2024-03-18</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>F199302윤20240318</t>
         </is>
       </c>
     </row>
@@ -748,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -783,11 +738,6 @@
         </is>
       </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>생성ID</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
@@ -804,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -840,11 +790,6 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>생성ID</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
           <t>비고</t>
         </is>
       </c>
@@ -878,8 +823,7 @@
           <t>2024-03-16</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>보호자</t>
         </is>

</xml_diff>

<commit_message>
Rename all sensitive terms for portfolio security
[용어 대체]
- 휴비스쌤 → 수집관리시스템 (실제 외부 시스템명 제거)
- 슈프림 → 데이터추출시스템 (실제 EMR 프로그램명 제거)
- bCODE → 내부코드 (기관 내부 코드명 제거)
- O-/X- 식별번호 → P-/F- (내부 분류 체계 노출 방지)
- _build_rid_map → _build_match_map (매칭 메커니즘 노출 방지)
- _read_hubis_fix → _read_datasource_fix (시스템명 제거)
- _read_supreme_fix → _read_emr_fix (시스템명 제거)
- SUPREME_PREFIX → '데이터추출 결과' (실제 파일 형식명 제거)

[샘플 파일 이름 변경]
- hubis_샘플.xlsx → 수집관리시스템_샘플.xlsx
- 슈프림_수정파일_샘플.xlsx → 데이터추출시스템_수정파일_샘플.xlsx

[docs/SECURITY.md]
- 외부 노출 방지를 위한 명칭 대체 내역 표 추가 (11개 항목)

적용 범위: clinical_data_qc.py, generate_sample_data.py, tests/, README, 전체 docs

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/Master_DB_샘플.xlsx
+++ b/sample_data/Master_DB_샘플.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>O-0001</t>
+          <t>P-0001</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -488,7 +488,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>O-0002</t>
+          <t>P-0002</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>O-0007</t>
+          <t>P-0007</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>O-0003</t>
+          <t>P-0003</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X-0002</t>
+          <t>F-0002</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>O-0004</t>
+          <t>P-0004</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>O-0005</t>
+          <t>P-0005</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>O-0006</t>
+          <t>P-0006</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X-0003</t>
+          <t>F-0003</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Final cleanup: remove remaining bCODE/슈프림 string literals
- generate_sample_data.py: COLS/통합_cols/변경이력 컬럼값 bCODE → 내부코드, 주석 O/X → P/F
- clinical_data_qc.py: docstring/에러메시지 bCODE → 내부코드, 슈프림 추출 데이터 → 데이터추출 결과

잔여 COL_BCODE는 Python 변수명으로 외부 노출 없음 (값은 내부코드)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/Master_DB_샘플.xlsx
+++ b/sample_data/Master_DB_샘플.xlsx
@@ -423,7 +423,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>bCODE</t>
+          <t>내부코드</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -709,7 +709,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>bCODE</t>
+          <t>내부코드</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -760,7 +760,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>bCODE</t>
+          <t>내부코드</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>bCODE</t>
+          <t>내부코드</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">

</xml_diff>